<commit_message>
Prepare corrected submission release v1.1.2
</commit_message>
<xml_diff>
--- a/code/portable_analysis/03_00_09_environment_lock/environment_manifest.xlsx
+++ b/code/portable_analysis/03_00_09_environment_lock/environment_manifest.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="1" r:id="Ra053e60aee1249ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input_Hashes" sheetId="2" r:id="R6f3ffd69fe124ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="1" r:id="R6456fc1501254aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input_Hashes" sheetId="2" r:id="R86092a4c0ec94ae1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -634,7 +634,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2579cc0053ff49a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7a5970c7de94ecc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1079,7 +1079,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1b6bf9e9eb34a3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7bc1375d2541cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>